<commit_message>
Week 6 Booked Hours
</commit_message>
<xml_diff>
--- a/Documentation/Week 6/Booked Hours/Booked_Hours_Dylan.xlsx
+++ b/Documentation/Week 6/Booked Hours/Booked_Hours_Dylan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24314441_student_uwa_edu_au/Documents/UWA/Year 3/Sem 2/CITS3200_Project/Documentation/Week 6/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="130" documentId="8_{C839D0D7-89B3-4B1F-A7FA-FAF46048CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{684EF329-DADD-4893-8492-631861C36E7C}"/>
+  <xr:revisionPtr revIDLastSave="131" documentId="8_{C839D0D7-89B3-4B1F-A7FA-FAF46048CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{977F3D22-AA9F-4603-939A-0D486ADC121B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="22">
   <si>
     <r>
       <t xml:space="preserve">CITS3200 Project Billed Hours Record for &lt;Dylan Hu&gt;
@@ -1459,6 +1459,9 @@
       <c r="E22" s="5">
         <v>0.98263888888888884</v>
       </c>
+      <c r="F22" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="G22" s="6">
         <f t="shared" si="0"/>
         <v>0.25000000011641532</v>

</xml_diff>